<commit_message>
menambahkan fitur upload gambar di buku_tamu
</commit_message>
<xml_diff>
--- a/laporan Buku Tamu.xlsx
+++ b/laporan Buku Tamu.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
   <si>
     <t>No</t>
   </si>
@@ -90,6 +90,21 @@
   </si>
   <si>
     <t>diffa</t>
+  </si>
+  <si>
+    <t>2026-09-24</t>
+  </si>
+  <si>
+    <t>tuya</t>
+  </si>
+  <si>
+    <t>btn</t>
+  </si>
+  <si>
+    <t>sasad</t>
+  </si>
+  <si>
+    <t>layangan</t>
   </si>
 </sst>
 </file>
@@ -429,7 +444,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -545,6 +560,29 @@
       </c>
       <c r="G5" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6">
+        <v>142131</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>